<commit_message>
Update tracking sheet with salary filter (>= R$5.000 or not informed)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01L34hAAD3zK3xkgXDX27zL1
</commit_message>
<xml_diff>
--- a/acompanhamento_candidaturas.xlsx
+++ b/acompanhamento_candidaturas.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O5"/>
+  <dimension ref="A1:O7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -526,7 +526,6 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
       <c r="B2" t="inlineStr">
         <is>
           <t>Arquiteto Pleno</t>
@@ -572,7 +571,6 @@
           <t>~19 dias (confirmar)</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr">
         <is>
           <t>A candidatar</t>
@@ -583,11 +581,8 @@
           <t>Confirmar se segue aberta</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr"/>
       <c r="B3" t="inlineStr">
         <is>
           <t>Arquiteto(a) de projetos</t>
@@ -633,7 +628,6 @@
           <t>?</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
           <t>A candidatar</t>
@@ -644,11 +638,8 @@
           <t>Localizar anúncio</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr"/>
       <c r="B4" t="inlineStr">
         <is>
           <t>Arquiteto</t>
@@ -694,7 +685,6 @@
           <t>?</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr">
         <is>
           <t>A candidatar</t>
@@ -705,11 +695,8 @@
           <t>Localizar anúncio</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
           <t>Arquiteto em Caruaru</t>
@@ -755,7 +742,6 @@
           <t>recente</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr">
         <is>
           <t>A candidatar</t>
@@ -766,8 +752,128 @@
           <t>Ver empresa e requisitos</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr"/>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Arquiteto (processo seletivo, 4 vagas)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Prefeitura de Ipojuca</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Ipojuca</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Site da prefeitura</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Contrato temporário</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>R$ 10.817,10</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Alta: exige CAU; análise de currículo e títulos</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>https://folha.qconcursos.com/n/prefeitura-de-ipojuca-pe-abre-processo-seletivo-com-8-vagas</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>~275 dias (provavelmente encerrado)</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Verificar se aberta</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Conferir edital no site da prefeitura</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr"/>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Engenheiro ou Arquiteto de Obras</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Método Potencial Engenharia</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Cabo de Santo Agostinho</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>JobLeads</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Temporário (~4 meses)</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Não informado</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Média/Alta: gestão de obras comerciais, 3 anos de experiência</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>https://www.jobleads.com/br/job/engenheiro-a-ou-arquiteto-a-de-obras-temporario-cabo-de-santo-agostinho-pe-legal-person--cabo-de-santo-agostinho--ee9856006001552014f6f95218797668a</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>~140 dias (pode estar fechada)</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Verificar se aberta</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Confirmar se segue aberta</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:O60"/>
@@ -789,7 +895,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -856,6 +962,30 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Filtro salarial</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Manter vagas com salário a partir de R$ 5.000 ou não informado; pular vagas abaixo de R$ 5.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Descartadas</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Arquiteto(a) de Legalizações Júnior, Consultoria Virtus RH, Cabo (R$ 600)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Recife openings to tracking sheet
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01L34hAAD3zK3xkgXDX27zL1
</commit_message>
<xml_diff>
--- a/acompanhamento_candidaturas.xlsx
+++ b/acompanhamento_candidaturas.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O7"/>
+  <dimension ref="A1:O11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -754,7 +754,6 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr">
         <is>
           <t>Arquiteto (processo seletivo, 4 vagas)</t>
@@ -800,7 +799,6 @@
           <t>~275 dias (provavelmente encerrado)</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
           <t>Verificar se aberta</t>
@@ -811,11 +809,8 @@
           <t>Conferir edital no site da prefeitura</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr"/>
       <c r="B7" t="inlineStr">
         <is>
           <t>Engenheiro ou Arquiteto de Obras</t>
@@ -861,7 +856,6 @@
           <t>~140 dias (pode estar fechada)</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr">
         <is>
           <t>Verificar se aberta</t>
@@ -872,8 +866,250 @@
           <t>Confirmar se segue aberta</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr"/>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Arquiteto projetista (liderança, aprovação na prefeitura)</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Vidor Real Estate</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Recife</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>BNE</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Efetivo, presencial</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>A combinar</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Alta: projetos de grandes edificações, AutoCAD, 3D, liderança</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>https://www.bne.com.br/vaga-de-emprego-na-area-construcao-em-recife-pe/arquiteto-projetista/4065191</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>verificar</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>A candidatar</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Confirmar se segue aberta; há também vaga da Vidor no Pina</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr"/>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Arquiteto</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>CALI TO</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Recife</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Agregador (Trabalha Brasil/BNE)</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>CLT ou PJ, presencial</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>R$ 5.000 + plano de saúde e ajuda de custo</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Média: piso do seu filtro</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>https://www.trabalhabrasil.com.br/vagas-de-emprego-em-recife-pe/arquiteto</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>verificar</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>A candidatar</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Localizar anúncio</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr"/>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Arquiteto de obras de varejo (gerenciar e fiscalizar)</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Não identificada</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Recife</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Catho</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Não informado</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Alta: arquitetura comercial/varejo</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>https://www.catho.com.br/vagas/arquiteto/recife-pe/</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>verificar</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>A candidatar</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Localizar anúncio e confirmar data</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr"/>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Coordenador de Projetos (remoto, não é só arquitetura)</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Grupo NRX</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Recife (remoto)</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Caderno Nacional</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>CLT</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>R$ 12.000 a 15.000</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Média: sua experiência como gerente de projetos</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>https://cadernonacional.com.br/vagas/coordenador-de-projetos/85613651</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>verificar</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>A candidatar</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Ver requisitos da área</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:O60"/>
@@ -895,7 +1131,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -986,6 +1222,18 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Descartadas (Recife)</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Direcional Engenharia, arquiteto de licenciamentos (R$ 3.395); Assistente de Projetos do Novo Atacarejo (nível assistente)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Caruaru opening, log discarded Recife/Caruaru roles
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01L34hAAD3zK3xkgXDX27zL1
</commit_message>
<xml_diff>
--- a/acompanhamento_candidaturas.xlsx
+++ b/acompanhamento_candidaturas.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O11"/>
+  <dimension ref="A1:O12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -868,7 +868,6 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr"/>
       <c r="B8" t="inlineStr">
         <is>
           <t>Arquiteto projetista (liderança, aprovação na prefeitura)</t>
@@ -914,7 +913,6 @@
           <t>verificar</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
           <t>A candidatar</t>
@@ -925,11 +923,8 @@
           <t>Confirmar se segue aberta; há também vaga da Vidor no Pina</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr"/>
       <c r="B9" t="inlineStr">
         <is>
           <t>Arquiteto</t>
@@ -975,7 +970,6 @@
           <t>verificar</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
           <t>A candidatar</t>
@@ -986,11 +980,8 @@
           <t>Localizar anúncio</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr"/>
       <c r="B10" t="inlineStr">
         <is>
           <t>Arquiteto de obras de varejo (gerenciar e fiscalizar)</t>
@@ -1036,7 +1027,6 @@
           <t>verificar</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr">
         <is>
           <t>A candidatar</t>
@@ -1047,11 +1037,8 @@
           <t>Localizar anúncio e confirmar data</t>
         </is>
       </c>
-      <c r="N10" t="inlineStr"/>
-      <c r="O10" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr">
         <is>
           <t>Coordenador de Projetos (remoto, não é só arquitetura)</t>
@@ -1097,7 +1084,6 @@
           <t>verificar</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr">
         <is>
           <t>A candidatar</t>
@@ -1108,8 +1094,67 @@
           <t>Ver requisitos da área</t>
         </is>
       </c>
-      <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr"/>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Arquiteto | Designer de Interiores (pleno/sênior, integral)</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Não identificada</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Caruaru</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>InfoJobs</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Não informado</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Alta: nível pleno/sênior</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>https://www.infojobs.com.br/vagas-de-arquiteto-em-caruaru,-pe.aspx</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>verificar</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>A candidatar</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Localizar anúncio (a página lista 14 vagas de arquiteto)</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:O60"/>
@@ -1131,7 +1176,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1234,6 +1279,18 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Descartadas (rodada 3)</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Recife: arquiteto R$ 2.800 (Fabiana Assunção); coordenação de curso (exige doutorado). Caruaru: Gestor de Projetos Estratégicos, CME Advogados (perfil de TI)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add senior/pleno Recife openings
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01L34hAAD3zK3xkgXDX27zL1
</commit_message>
<xml_diff>
--- a/acompanhamento_candidaturas.xlsx
+++ b/acompanhamento_candidaturas.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O12"/>
+  <dimension ref="A1:O14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1096,7 +1096,6 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
           <t>Arquiteto | Designer de Interiores (pleno/sênior, integral)</t>
@@ -1142,7 +1141,6 @@
           <t>verificar</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr">
         <is>
           <t>A candidatar</t>
@@ -1153,8 +1151,128 @@
           <t>Localizar anúncio (a página lista 14 vagas de arquiteto)</t>
         </is>
       </c>
-      <c r="N12" t="inlineStr"/>
-      <c r="O12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr"/>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Arquiteto (residencial e comercial, compatibilização, aprovação)</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Grupo Referencial</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Recife</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Glassdoor/agregadores</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Não informado</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Alta: AutoCAD, SketchUp, Revit; projetos comerciais</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>https://www.glassdoor.com.br/Vaga/recife-arquiteto-vagas-SRCH_IL.0,6_IC2504041_KO7,16.htm</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>verificar</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>A candidatar</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Localizar anúncio</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr"/>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Analista de Projetos - PE</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Moura Dubeux</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Recife</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Não informado</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Média: incorporadora; confirmar se a função é de arquitetura</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>https://br.linkedin.com/jobs/arquiteto-vagas-recife</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>~1 semana (visto na listagem)</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>Verificar</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>Ver descrição e salário no LinkedIn</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr"/>
+      <c r="O14" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:O60"/>
@@ -1176,7 +1294,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1291,6 +1409,18 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Nota Eddios</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Anúncio em agregador (abril/2026): R$ 6.000 a 7.200, CLT, 6h por dia, Revit e AutoCAD</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add editais e órgãos sheet (perícias e avaliações)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01L34hAAD3zK3xkgXDX27zL1
</commit_message>
<xml_diff>
--- a/acompanhamento_candidaturas.xlsx
+++ b/acompanhamento_candidaturas.xlsx
@@ -9,9 +9,11 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Candidaturas" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Perfil e buscas" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Editais e órgãos" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Candidaturas'!$A$1:$O$60</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Editais e órgãos'!$A$1:$K$40</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -58,10 +60,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1153,7 +1158,6 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr"/>
       <c r="B13" t="inlineStr">
         <is>
           <t>Arquiteto (residencial e comercial, compatibilização, aprovação)</t>
@@ -1199,7 +1203,6 @@
           <t>verificar</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr">
         <is>
           <t>A candidatar</t>
@@ -1210,11 +1213,8 @@
           <t>Localizar anúncio</t>
         </is>
       </c>
-      <c r="N13" t="inlineStr"/>
-      <c r="O13" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr"/>
       <c r="B14" t="inlineStr">
         <is>
           <t>Analista de Projetos - PE</t>
@@ -1260,7 +1260,6 @@
           <t>~1 semana (visto na listagem)</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr">
         <is>
           <t>Verificar</t>
@@ -1271,8 +1270,6 @@
           <t>Ver descrição e salário no LinkedIn</t>
         </is>
       </c>
-      <c r="N14" t="inlineStr"/>
-      <c r="O14" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:O60"/>
@@ -1424,4 +1421,571 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
+    <col width="44" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="44" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="36" customWidth="1" min="10" max="10"/>
+    <col width="40" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Órgão / Edital</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Região</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>O que fazer</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Documentos / requisitos</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Situação</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Prazo</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Próximo passo</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal, Edital de Credenciamento nº 012/2026</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Banco, avaliação de imóveis</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Nacional</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Acompanhar andamento</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Registro CAU; foco do edital: empresas precificadoras (AVM, sem vistoria)</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>https://caubr.gov.br/cau-br-apresenta-impugnacao-ao-edital-de-credenciamento-da-caixa/</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Contestado pelo CAU/BR, CREA-SC e Confea; mandado de segurança. Republicado em 30/01/2026. Situação atual não confirmada</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Verificar</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Conferir no Portal de Licitações da Caixa se foi suspenso ou mantido</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Formato pode não atender pessoa física com vistoria</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Caixa, credenciamento tradicional de avaliadores (modelo edital 0244/2024)</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Banco, avaliação de imóveis</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Nacional</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Aguardar novo edital e preparar documentos</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Registro CREA/CAU; certidão de acervo técnico de avaliações; ABNT NBR 14.653</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>https://roteirodepericias.com.br/2024/04/11/caixa-abre-cadastramento-de-avaliadores-de-imoveis/</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Edital de 2024; prazos de novos editais costumam ser curtos</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Aguardar</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Reunir documentos antes do novo edital</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>Currículo não cita avaliações: confirmar com o CAU-PE como comprovar experiência</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>TJPE, cadastro CPTEC (SIAJUS)</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Justiça estadual, perícias judiciais</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Caruaru e comarcas do TJPE</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Inscrição no portal de auxiliares da justiça (pessoa física)</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Registro ativo no CAU; documentos pessoais e formação</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>https://portal.tjpe.jus.br/web/transparencia/gestao-de-pessoas/peritos-e-orgaos-tecnicos-ou-cientificos</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Cadastro permanente; confirmar período de inscrição</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Verificar</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Ler requisitos completos e inscrever-se</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>Peritos são nomeados entre os inscritos</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>TRF5 / Justiça Federal, sistema AJG/JF</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Justiça Federal, perícias</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Pernambuco (JFPE)</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Cadastro no AJG/JF</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Registro no CAU; curso de perícia de engenharia do CJF (vícios em imóveis MCMV Faixa 1, Recomendação 3/2025)</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>https://www.trf5.jus.br/index.php/noticias/leitura-de-noticias?%2Fid=324889</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Cadastro permanente</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Verificar</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Verificar o curso do CJF e a inscrição</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>Ações do Minha Casa, Minha Vida exigem o curso</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Ministério da Gestão (SPU), credenciamento de avaliadores de imóveis</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Governo federal</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Nacional</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Conferir se há chamamento aberto</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>A confirmar na página do órgão</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.gov.br/gestao/pt-br/federativo/programa-nacional-de-gestao-e-inovacao/credenciamento_de_avaliadores_de_imoveis</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Não confirmada</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Verificar</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Ler a página e checar chamamentos</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Editais de credenciamento em bancos (agregador Laudo Master)</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Bancos</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Nacional</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Acompanhar editais de BB, Bradesco, Caixa e outros</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Registro CAU; NBR 14.653</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>https://laudomaster.com.br/editais/</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Lista de editais; verificar o que está aberto</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Verificar</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Abrir a página e filtrar os abertos</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>MPPE e Defensoria Pública de Pernambuco</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Ministério Público / Defensoria</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Pernambuco</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Verificar editais de credenciamento de peritos</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>A confirmar</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr"/>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Não encontrado pela busca</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Verificar</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Consultar os sites de cada órgão</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>Referência: MPMG abriu o Edital 001/2026 em Minas</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Prefeituras do Agreste (Caruaru, Gravatá, Bezerros, Santa Cruz do Capibaribe)</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Prefeituras</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Caruaru e vizinhas</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Verificar credenciamento ou dispensa para laudos e avaliações</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>A confirmar</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr"/>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Não encontrado pela busca</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Verificar</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Consultar portais da transparência e Diário Oficial dos municípios</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>CAU-PE</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Conselho profissional</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Pernambuco</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Perguntar sobre registro, acervo técnico e vagas de avaliação</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Registro ativo CAU-PE A166156-6</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr"/>
+      <c r="G10" s="2" t="inlineStr"/>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Verificar</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr"/>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Contato com a comissão competente</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:K40"/>
+  <dataValidations count="1">
+    <dataValidation sqref="H2:H40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Verificar,Aguardar,Em preparação,Inscrito,Credenciado,Descartado"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>